<commit_message>
updated sarcasm detection model, updated with reran data
</commit_message>
<xml_diff>
--- a/data/pipeline_latency_summary.xlsx
+++ b/data/pipeline_latency_summary.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,37 +417,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>run</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>records</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>elapsed_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>records_per_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>s_per_record</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -477,16 +465,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>369</v>
+        <v>396</v>
       </c>
       <c r="D2" t="n">
-        <v>30.9015</v>
+        <v>29.4864</v>
       </c>
       <c r="E2" t="n">
-        <v>11.9412</v>
+        <v>13.4299</v>
       </c>
       <c r="F2" t="n">
-        <v>0.083744</v>
+        <v>0.074461</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -502,16 +490,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>547</v>
+        <v>604</v>
       </c>
       <c r="D3" t="n">
-        <v>99.1901</v>
+        <v>73.8357</v>
       </c>
       <c r="E3" t="n">
-        <v>5.5147</v>
+        <v>8.180300000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>0.181335</v>
+        <v>0.122245</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
@@ -527,16 +515,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>916</v>
+        <v>1000</v>
       </c>
       <c r="D4" t="n">
-        <v>130.0916</v>
+        <v>103.3221</v>
       </c>
       <c r="E4" t="n">
-        <v>7.0412</v>
+        <v>9.6785</v>
       </c>
       <c r="F4" t="n">
-        <v>0.142021</v>
+        <v>0.103322</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ran classification for full dataset
</commit_message>
<xml_diff>
--- a/data/pipeline_latency_summary.xlsx
+++ b/data/pipeline_latency_summary.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,41 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>run</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>records</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>elapsed_s</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>records_per_s</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>s_per_record</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -461,20 +473,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RoBERTa (overall)</t>
+          <t>Subjectivity — GroNLP model</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>396</v>
+        <v>7796</v>
       </c>
       <c r="D2" t="n">
-        <v>29.4864</v>
+        <v>1342.6579</v>
       </c>
       <c r="E2" t="n">
-        <v>13.4299</v>
+        <v>5.8064</v>
       </c>
       <c r="F2" t="n">
-        <v>0.074461</v>
+        <v>0.172224</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -486,20 +498,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DeBERTa-base-finetuned ABSA (aspect)</t>
+          <t>Subjectivity — SenticNet fallback</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>604</v>
+        <v>4331</v>
       </c>
       <c r="D3" t="n">
-        <v>73.8357</v>
+        <v>0.6473</v>
       </c>
       <c r="E3" t="n">
-        <v>8.180300000000001</v>
+        <v>6690.8698</v>
       </c>
       <c r="F3" t="n">
-        <v>0.122245</v>
+        <v>0.000149</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
@@ -511,22 +523,97 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Sarcasm detection</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7796</v>
+      </c>
+      <c r="D4" t="n">
+        <v>659.4837</v>
+      </c>
+      <c r="E4" t="n">
+        <v>11.8214</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.084593</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Run5_RoBERTa_DeBERTaBase_finetuned_subjectivity_hybrid_sarcasm</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RoBERTa (overall)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2883</v>
+      </c>
+      <c r="D5" t="n">
+        <v>269.6139</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10.6931</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.093519</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Run5_RoBERTa_DeBERTaBase_finetuned_subjectivity_hybrid_sarcasm</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DeBERTa-base-finetuned ABSA (aspect)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4140</v>
+      </c>
+      <c r="D6" t="n">
+        <v>669.9773</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6.1793</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.16183</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Run5_RoBERTa_DeBERTaBase_finetuned_subjectivity_hybrid_sarcasm</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>TOTAL (all model stages)</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D4" t="n">
-        <v>103.3221</v>
-      </c>
-      <c r="E4" t="n">
-        <v>9.6785</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.103322</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="C7" t="n">
+        <v>26946</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2942.3801</v>
+      </c>
+      <c r="E7" t="n">
+        <v>9.1579</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.109195</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>excludes objective rows (rule-assigned neutral, no model time)</t>
         </is>

</xml_diff>